<commit_message>
Add finance import tools and populate tracker
- Airbnb CSV import skill + script (auto-detect, dedup, stub enrichment)
- Bank statement import script (Robinhood CC categorization with vendor map)
- Mileage log generator (reconstructs trips from CC location data)
- Finance tracker: 4 bookings, 69 expenses, 20-trip mileage log
- Dashboard HTML for visual finance overview
</commit_message>
<xml_diff>
--- a/finances/kengs-landing-finance-tracker.xlsx
+++ b/finances/kengs-landing-finance-tracker.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment &amp; ROI" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget vs Actual" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category Reference" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mileage Log" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bookings'!$A$1:$L$101</definedName>
@@ -24,11 +25,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="168" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -111,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -120,20 +122,28 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -615,23 +625,43 @@
           <t>Apr 2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Tyler Nicholson</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>46114</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>46118</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>127.32</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>75</v>
+      </c>
       <c r="I3" s="4" t="n">
-        <v>590.97</v>
-      </c>
-      <c r="J3" s="4" t="n"/>
+        <v>609.27</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>18.3</v>
+      </c>
       <c r="K3" s="4" t="n">
         <v>590.97</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Payout received 2026-04-06 — platform TBD</t>
+          <t>Airbnb HMTK9FNMQK | Pet fee: $25.00 | Tax remitted: $40.05</t>
         </is>
       </c>
     </row>
@@ -641,23 +671,43 @@
           <t>Apr 2026</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Kepi Garner Jr</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>46118</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>46120</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>124.81</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>75</v>
+      </c>
       <c r="I4" s="4" t="n">
-        <v>314.86</v>
-      </c>
-      <c r="J4" s="4" t="n"/>
+        <v>324.61</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>9.75</v>
+      </c>
       <c r="K4" s="4" t="n">
         <v>314.86</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Payout received 2026-04-08 — platform TBD</t>
+          <t>Airbnb HMRWNBH82B | Tax remitted: $21.34</t>
         </is>
       </c>
     </row>
@@ -667,23 +717,41 @@
           <t>Apr 2026</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="4" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Dalyce Sellers</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>46122</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>46126</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>105.2</v>
+      </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n">
-        <v>408.18</v>
-      </c>
-      <c r="J5" s="4" t="n"/>
+        <v>420.8</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>12.62</v>
+      </c>
       <c r="K5" s="4" t="n">
         <v>408.18</v>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Payout received 2026-04-17 — platform TBD</t>
+          <t>Airbnb HM4MWDKA2D | Tax remitted: $25.25</t>
         </is>
       </c>
     </row>
@@ -2220,927 +2288,2511 @@
       <c r="I4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
+      <c r="A5" s="3" t="n">
+        <v>46023</v>
+      </c>
       <c r="B5" s="2">
         <f>IF(A5="","",TEXT(A5,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Lowe's</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>LOWES #00907* 866-483-7521 NC | Dishwasher</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>323.67</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
+      <c r="A6" s="3" t="n">
+        <v>46023</v>
+      </c>
       <c r="B6" s="2">
         <f>IF(A6="","",TEXT(A6,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Brookshire Brothers</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>BROOKSHIRE BROS #10 FAIRFIELD TX | Property supplies</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>12.06</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
+      <c r="A7" s="3" t="n">
+        <v>46025</v>
+      </c>
       <c r="B7" s="2">
         <f>IF(A7="","",TEXT(A7,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Dfw Estate Liquidators</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>DFW ESTATE LIQUIDATORS WEATHERFORD TX | Furnishing</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>48.46</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
+      <c r="A8" s="3" t="n">
+        <v>46025</v>
+      </c>
       <c r="B8" s="2">
         <f>IF(A8="","",TEXT(A8,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Dfw Estate Liquidators</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>DFW ESTATE LIQUIDATORS WEATHERFORD TX | Furnishing</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
+      <c r="A9" s="3" t="n">
+        <v>46026</v>
+      </c>
       <c r="B9" s="2">
         <f>IF(A9="","",TEXT(A9,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>-20.92</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
+      <c r="A10" s="3" t="n">
+        <v>46026</v>
+      </c>
       <c r="B10" s="2">
         <f>IF(A10="","",TEXT(A10,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>-17.47</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
+      <c r="A11" s="3" t="n">
+        <v>46027</v>
+      </c>
       <c r="B11" s="2">
         <f>IF(A11="","",TEXT(A11,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>269.82</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
+      <c r="A12" s="3" t="n">
+        <v>46028</v>
+      </c>
       <c r="B12" s="2">
         <f>IF(A12="","",TEXT(A12,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Maga Waste, Llc</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>TRB MAGA WASTE LLC 802-5603595 VT | Trash service</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>170</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
+      <c r="A13" s="3" t="n">
+        <v>46029</v>
+      </c>
       <c r="B13" s="2">
         <f>IF(A13="","",TEXT(A13,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #6568 MANSFIELD TX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>142.7</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n"/>
+      <c r="A14" s="3" t="n">
+        <v>46031</v>
+      </c>
       <c r="B14" s="2">
         <f>IF(A14="","",TEXT(A14,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Burger King</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - Burger King | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>20.56</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n"/>
+      <c r="A15" s="3" t="n">
+        <v>46031</v>
+      </c>
       <c r="B15" s="2">
         <f>IF(A15="","",TEXT(A15,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Brookshire Brothers</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>BROOKSHIRE BROS #10 FAIRFIELD TX | Property supplies</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>43.42</v>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n"/>
+      <c r="A16" s="3" t="n">
+        <v>46031</v>
+      </c>
       <c r="B16" s="2">
         <f>IF(A16="","",TEXT(A16,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>32.02</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n"/>
+      <c r="A17" s="3" t="n">
+        <v>46032</v>
+      </c>
       <c r="B17" s="2">
         <f>IF(A17="","",TEXT(A17,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>142.12</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n"/>
+      <c r="A18" s="3" t="n">
+        <v>46032</v>
+      </c>
       <c r="B18" s="2">
         <f>IF(A18="","",TEXT(A18,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>17.97</v>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n"/>
+      <c r="A19" s="3" t="n">
+        <v>46034</v>
+      </c>
       <c r="B19" s="2">
         <f>IF(A19="","",TEXT(A19,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>-20.46</v>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n"/>
+      <c r="A20" s="3" t="n">
+        <v>46034</v>
+      </c>
       <c r="B20" s="2">
         <f>IF(A20="","",TEXT(A20,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>-119.92</v>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n"/>
+      <c r="A21" s="3" t="n">
+        <v>46035</v>
+      </c>
       <c r="B21" s="2">
         <f>IF(A21="","",TEXT(A21,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>HOMEDEPOT.COM 800-430-3376 GA | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>269</v>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n"/>
+      <c r="A22" s="3" t="n">
+        <v>46035</v>
+      </c>
       <c r="B22" s="2">
         <f>IF(A22="","",TEXT(A22,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>HOMEDEPOT.COM 800-430-3376 GA | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>46.12</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n"/>
+      <c r="A23" s="3" t="n">
+        <v>46037</v>
+      </c>
       <c r="B23" s="2">
         <f>IF(A23="","",TEXT(A23,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>1066.5</v>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n"/>
+      <c r="A24" s="3" t="n">
+        <v>46037</v>
+      </c>
       <c r="B24" s="2">
         <f>IF(A24="","",TEXT(A24,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Brenco</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>BRENCO FAIRFIELD TX</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>74.23</v>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n"/>
+      <c r="A25" s="3" t="n">
+        <v>46038</v>
+      </c>
       <c r="B25" s="2">
         <f>IF(A25="","",TEXT(A25,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>486.62</v>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n"/>
+      <c r="A26" s="3" t="n">
+        <v>46039</v>
+      </c>
       <c r="B26" s="2">
         <f>IF(A26="","",TEXT(A26,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Brookshire Brothers</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>BROOKSHIRE BROS #10 FAIRFIELD TX | Property supplies</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>102.63</v>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n"/>
+      <c r="A27" s="3" t="n">
+        <v>46040</v>
+      </c>
       <c r="B27" s="2">
         <f>IF(A27="","",TEXT(A27,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Ace Home Center</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>ACE HOME CENTER FAIRFIELD TX</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>8.65</v>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n"/>
+      <c r="A28" s="3" t="n">
+        <v>46040</v>
+      </c>
       <c r="B28" s="2">
         <f>IF(A28="","",TEXT(A28,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Pizza Hut</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - Pizza Hut | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>24.13</v>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n"/>
+      <c r="A29" s="3" t="n">
+        <v>46042</v>
+      </c>
       <c r="B29" s="2">
         <f>IF(A29="","",TEXT(A29,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>601</v>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n"/>
+      <c r="A30" s="3" t="n">
+        <v>46042</v>
+      </c>
       <c r="B30" s="2">
         <f>IF(A30="","",TEXT(A30,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>-269</v>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n"/>
+      <c r="A31" s="3" t="n">
+        <v>46042</v>
+      </c>
       <c r="B31" s="2">
         <f>IF(A31="","",TEXT(A31,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>14.98</v>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n"/>
+      <c r="A32" s="3" t="n">
+        <v>46042</v>
+      </c>
       <c r="B32" s="2">
         <f>IF(A32="","",TEXT(A32,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #0507 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>68.95999999999999</v>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n"/>
+      <c r="A33" s="3" t="n">
+        <v>46048</v>
+      </c>
       <c r="B33" s="2">
         <f>IF(A33="","",TEXT(A33,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Gexa Energy</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>GEXA ENERGY 866-329-4392 TX | Electric</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>81.89</v>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n"/>
+      <c r="A34" s="3" t="n">
+        <v>46057</v>
+      </c>
       <c r="B34" s="2">
         <f>IF(A34="","",TEXT(A34,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="4" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #6568 MANSFIELD TX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n"/>
+      <c r="A35" s="3" t="n">
+        <v>46057</v>
+      </c>
       <c r="B35" s="2">
         <f>IF(A35="","",TEXT(A35,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #6568 MANSFIELD TX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>-35.98</v>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="n"/>
+      <c r="A36" s="3" t="n">
+        <v>46060</v>
+      </c>
       <c r="B36" s="2">
         <f>IF(A36="","",TEXT(A36,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Capps True Value Hardware and Ag Center</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>CAPPS TRUE VALUE FAIRFIELD TX</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>14.07</v>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n"/>
+      <c r="A37" s="3" t="n">
+        <v>46061</v>
+      </c>
       <c r="B37" s="2">
         <f>IF(A37="","",TEXT(A37,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>HOMEDEPOT.COM 800-430-3376 GA | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>39.98</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n"/>
+      <c r="A38" s="3" t="n">
+        <v>46063</v>
+      </c>
       <c r="B38" s="2">
         <f>IF(A38="","",TEXT(A38,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>-449</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n"/>
+      <c r="A39" s="3" t="n">
+        <v>46063</v>
+      </c>
       <c r="B39" s="2">
         <f>IF(A39="","",TEXT(A39,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>-373</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n"/>
+      <c r="A40" s="3" t="n">
+        <v>46063</v>
+      </c>
       <c r="B40" s="2">
         <f>IF(A40="","",TEXT(A40,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>-69.95999999999999</v>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I40" s="2" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n"/>
+      <c r="A41" s="3" t="n">
+        <v>46063</v>
+      </c>
       <c r="B41" s="2">
         <f>IF(A41="","",TEXT(A41,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="2" t="n"/>
-      <c r="H41" s="2" t="n"/>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT 6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>281.82</v>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="n"/>
+      <c r="A42" s="3" t="n">
+        <v>46067</v>
+      </c>
       <c r="B42" s="2">
         <f>IF(A42="","",TEXT(A42,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="4" t="n"/>
-      <c r="G42" s="2" t="n"/>
-      <c r="H42" s="2" t="n"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Wendy's</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - Wendy's | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n"/>
+      <c r="A43" s="3" t="n">
+        <v>46069</v>
+      </c>
       <c r="B43" s="2">
         <f>IF(A43="","",TEXT(A43,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="2" t="n"/>
-      <c r="H43" s="2" t="n"/>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>-111.06</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="n"/>
+      <c r="A44" s="3" t="n">
+        <v>46069</v>
+      </c>
       <c r="B44" s="2">
         <f>IF(A44="","",TEXT(A44,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="2" t="n"/>
-      <c r="H44" s="2" t="n"/>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>-159</v>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="n"/>
+      <c r="A45" s="3" t="n">
+        <v>46069</v>
+      </c>
       <c r="B45" s="2">
         <f>IF(A45="","",TEXT(A45,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="2" t="n"/>
-      <c r="H45" s="2" t="n"/>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>-24.82</v>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="n"/>
+      <c r="A46" s="3" t="n">
+        <v>46076</v>
+      </c>
       <c r="B46" s="2">
         <f>IF(A46="","",TEXT(A46,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="2" t="n"/>
-      <c r="H46" s="2" t="n"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Gexa Energy</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>GEXA ENERGY 866-329-4392 TX | Electric</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="n"/>
+      <c r="A47" s="3" t="n">
+        <v>46079</v>
+      </c>
       <c r="B47" s="2">
         <f>IF(A47="","",TEXT(A47,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="2" t="n"/>
-      <c r="H47" s="2" t="n"/>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>HOMEDEPOT.COM 800-430-3376 GA | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>199</v>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="n"/>
+      <c r="A48" s="3" t="n">
+        <v>46084</v>
+      </c>
       <c r="B48" s="2">
         <f>IF(A48="","",TEXT(A48,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C48" s="2" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="4" t="n"/>
-      <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="n"/>
+      <c r="A49" s="3" t="n">
+        <v>46084</v>
+      </c>
       <c r="B49" s="2">
         <f>IF(A49="","",TEXT(A49,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="2" t="n"/>
-      <c r="H49" s="2" t="n"/>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>-114.21</v>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="n"/>
+      <c r="A50" s="3" t="n">
+        <v>46085</v>
+      </c>
       <c r="B50" s="2">
         <f>IF(A50="","",TEXT(A50,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="2" t="n"/>
-      <c r="H50" s="2" t="n"/>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Love's Travel Stop</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - Love's Travel Stop | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>70.43000000000001</v>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I50" s="2" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="n"/>
+      <c r="A51" s="3" t="n">
+        <v>46090</v>
+      </c>
       <c r="B51" s="2">
         <f>IF(A51="","",TEXT(A51,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C51" s="2" t="n"/>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="2" t="n"/>
-      <c r="H51" s="2" t="n"/>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Brookshire Brothers</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>BROOKSHIRE BROS #10 FAIRFIELD TX | Property supplies</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>149.49</v>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I51" s="2" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="n"/>
+      <c r="A52" s="3" t="n">
+        <v>46090</v>
+      </c>
       <c r="B52" s="2">
         <f>IF(A52="","",TEXT(A52,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C52" s="2" t="n"/>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="4" t="n"/>
-      <c r="G52" s="2" t="n"/>
-      <c r="H52" s="2" t="n"/>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Ace Home Center</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>ACE HOME CENTER FAIRFIELD TX</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>59.57</v>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="n"/>
+      <c r="A53" s="3" t="n">
+        <v>46098</v>
+      </c>
       <c r="B53" s="2">
         <f>IF(A53="","",TEXT(A53,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C53" s="2" t="n"/>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="4" t="n"/>
-      <c r="G53" s="2" t="n"/>
-      <c r="H53" s="2" t="n"/>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Ace Home Center</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>ACE HOME CENTER FAIRFIELD TX</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>19.98</v>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="n"/>
+      <c r="A54" s="3" t="n">
+        <v>46100</v>
+      </c>
       <c r="B54" s="2">
         <f>IF(A54="","",TEXT(A54,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C54" s="2" t="n"/>
-      <c r="D54" s="2" t="n"/>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="2" t="n"/>
-      <c r="H54" s="2" t="n"/>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>El Jimador Mexican Grill 7</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - El Jimador Mexican Grill 7 | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="n"/>
+      <c r="A55" s="3" t="n">
+        <v>46101</v>
+      </c>
       <c r="B55" s="2">
         <f>IF(A55="","",TEXT(A55,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C55" s="2" t="n"/>
-      <c r="D55" s="2" t="n"/>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="2" t="n"/>
-      <c r="H55" s="2" t="n"/>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>REFUND: THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>-114.35</v>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="n"/>
+      <c r="A56" s="3" t="n">
+        <v>46101</v>
+      </c>
       <c r="B56" s="2">
         <f>IF(A56="","",TEXT(A56,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C56" s="2" t="n"/>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="4" t="n"/>
-      <c r="G56" s="2" t="n"/>
-      <c r="H56" s="2" t="n"/>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Gulf</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - Gulf | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>68.84</v>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I56" s="2" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="n"/>
+      <c r="A57" s="3" t="n">
+        <v>46106</v>
+      </c>
       <c r="B57" s="2">
         <f>IF(A57="","",TEXT(A57,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C57" s="2" t="n"/>
-      <c r="D57" s="2" t="n"/>
-      <c r="E57" s="2" t="n"/>
-      <c r="F57" s="4" t="n"/>
-      <c r="G57" s="2" t="n"/>
-      <c r="H57" s="2" t="n"/>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Braum's</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - Braum's | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I57" s="2" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="n"/>
+      <c r="A58" s="3" t="n">
+        <v>46106</v>
+      </c>
       <c r="B58" s="2">
         <f>IF(A58="","",TEXT(A58,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C58" s="2" t="n"/>
-      <c r="D58" s="2" t="n"/>
-      <c r="E58" s="2" t="n"/>
-      <c r="F58" s="4" t="n"/>
-      <c r="G58" s="2" t="n"/>
-      <c r="H58" s="2" t="n"/>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Braum's</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - Braum's | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="n"/>
+      <c r="A59" s="3" t="n">
+        <v>46107</v>
+      </c>
       <c r="B59" s="2">
         <f>IF(A59="","",TEXT(A59,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C59" s="2" t="n"/>
-      <c r="D59" s="2" t="n"/>
-      <c r="E59" s="2" t="n"/>
-      <c r="F59" s="4" t="n"/>
-      <c r="G59" s="2" t="n"/>
-      <c r="H59" s="2" t="n"/>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Gexa Energy</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>GEXA ENERGY 866-329-4392 TX | Electric</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>140.3</v>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I59" s="2" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="n"/>
+      <c r="A60" s="3" t="n">
+        <v>46107</v>
+      </c>
       <c r="B60" s="2">
         <f>IF(A60="","",TEXT(A60,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C60" s="2" t="n"/>
-      <c r="D60" s="2" t="n"/>
-      <c r="E60" s="2" t="n"/>
-      <c r="F60" s="4" t="n"/>
-      <c r="G60" s="2" t="n"/>
-      <c r="H60" s="2" t="n"/>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>North Texas Tollway Authority</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>NTTA ONLINE 972-818-6882 TX | Tolls for property trips</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I60" s="2" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="n"/>
+      <c r="A61" s="3" t="n">
+        <v>46109</v>
+      </c>
       <c r="B61" s="2">
         <f>IF(A61="","",TEXT(A61,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C61" s="2" t="n"/>
-      <c r="D61" s="2" t="n"/>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="4" t="n"/>
-      <c r="G61" s="2" t="n"/>
-      <c r="H61" s="2" t="n"/>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Discount Tire</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>DISCOUNT-TIRE-CO TXD-64 MANSFIELD TX | Tire replacement from property trips</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>214.58</v>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I61" s="2" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="n"/>
+      <c r="A62" s="3" t="n">
+        <v>46112</v>
+      </c>
       <c r="B62" s="2">
         <f>IF(A62="","",TEXT(A62,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C62" s="2" t="n"/>
-      <c r="D62" s="2" t="n"/>
-      <c r="E62" s="2" t="n"/>
-      <c r="F62" s="4" t="n"/>
-      <c r="G62" s="2" t="n"/>
-      <c r="H62" s="2" t="n"/>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Professional Services</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Intuit</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>INTUIT *TURBOTAX 800-446-8848 CA | TurboTax (prorate STR %)</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="n"/>
+      <c r="A63" s="3" t="n">
+        <v>46113</v>
+      </c>
       <c r="B63" s="2">
         <f>IF(A63="","",TEXT(A63,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C63" s="2" t="n"/>
-      <c r="D63" s="2" t="n"/>
-      <c r="E63" s="2" t="n"/>
-      <c r="F63" s="4" t="n"/>
-      <c r="G63" s="2" t="n"/>
-      <c r="H63" s="2" t="n"/>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Taco Bell</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - Taco Bell | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I63" s="2" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n"/>
+      <c r="A64" s="3" t="n">
+        <v>46113</v>
+      </c>
       <c r="B64" s="2">
         <f>IF(A64="","",TEXT(A64,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C64" s="2" t="n"/>
-      <c r="D64" s="2" t="n"/>
-      <c r="E64" s="2" t="n"/>
-      <c r="F64" s="4" t="n"/>
-      <c r="G64" s="2" t="n"/>
-      <c r="H64" s="2" t="n"/>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - Shell | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="n">
+        <v>61.19</v>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I64" s="2" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="n"/>
+      <c r="A65" s="3" t="n">
+        <v>46113</v>
+      </c>
       <c r="B65" s="2">
         <f>IF(A65="","",TEXT(A65,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C65" s="2" t="n"/>
-      <c r="D65" s="2" t="n"/>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="4" t="n"/>
-      <c r="G65" s="2" t="n"/>
-      <c r="H65" s="2" t="n"/>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #6817 CORSICANA TX</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>19.74</v>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I65" s="2" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="n"/>
+      <c r="A66" s="3" t="n">
+        <v>46114</v>
+      </c>
       <c r="B66" s="2">
         <f>IF(A66="","",TEXT(A66,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C66" s="2" t="n"/>
-      <c r="D66" s="2" t="n"/>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="4" t="n"/>
-      <c r="G66" s="2" t="n"/>
-      <c r="H66" s="2" t="n"/>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Brookshire Brothers</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>BROOKSHIRE BROS #10 FAIRFIELD TX | Property supplies</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>39.44</v>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I66" s="2" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="n"/>
+      <c r="A67" s="3" t="n">
+        <v>46114</v>
+      </c>
       <c r="B67" s="2">
         <f>IF(A67="","",TEXT(A67,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C67" s="2" t="n"/>
-      <c r="D67" s="2" t="n"/>
-      <c r="E67" s="2" t="n"/>
-      <c r="F67" s="4" t="n"/>
-      <c r="G67" s="2" t="n"/>
-      <c r="H67" s="2" t="n"/>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Brookshire Brothers</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>BROOKSHIRE BROS #10 FAIRFIELD TX | Property supplies</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>69.77</v>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I67" s="2" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="n"/>
+      <c r="A68" s="3" t="n">
+        <v>46114</v>
+      </c>
       <c r="B68" s="2">
         <f>IF(A68="","",TEXT(A68,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C68" s="2" t="n"/>
-      <c r="D68" s="2" t="n"/>
-      <c r="E68" s="2" t="n"/>
-      <c r="F68" s="4" t="n"/>
-      <c r="G68" s="2" t="n"/>
-      <c r="H68" s="2" t="n"/>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Cooper Farms</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>COOPER FARMS COUNTRY STORFAIRFIELD TX</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I68" s="2" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="n"/>
+      <c r="A69" s="3" t="n">
+        <v>46114</v>
+      </c>
       <c r="B69" s="2">
         <f>IF(A69="","",TEXT(A69,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C69" s="2" t="n"/>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="n"/>
-      <c r="F69" s="4" t="n"/>
-      <c r="G69" s="2" t="n"/>
-      <c r="H69" s="2" t="n"/>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Travel / Mileage</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Burger King</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Travel meals/fuel - Burger King | Trip to Fairfield</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>5.41</v>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I69" s="2" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="n"/>
+      <c r="A70" s="3" t="n">
+        <v>46118</v>
+      </c>
       <c r="B70" s="2">
         <f>IF(A70="","",TEXT(A70,"MMM YYYY"))</f>
         <v/>
       </c>
-      <c r="C70" s="2" t="n"/>
-      <c r="D70" s="2" t="n"/>
-      <c r="E70" s="2" t="n"/>
-      <c r="F70" s="4" t="n"/>
-      <c r="G70" s="2" t="n"/>
-      <c r="H70" s="2" t="n"/>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>THE HOME DEPOT #8517 GRAND PRAIRIETX | VERIFY: GP/Mansfield HD - STR or personal?</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="n">
+        <v>69.75</v>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Robinhood CC</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I70" s="2" t="n"/>
     </row>
     <row r="71">
@@ -5020,7 +6672,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -5084,7 +6735,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A4)</f>
         <v/>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="20">
         <f>IFERROR(F4/31,0)</f>
         <v/>
       </c>
@@ -5115,7 +6766,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A5)</f>
         <v/>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="20">
         <f>IFERROR(F5/28,0)</f>
         <v/>
       </c>
@@ -5146,7 +6797,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A6)</f>
         <v/>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="20">
         <f>IFERROR(F6/31,0)</f>
         <v/>
       </c>
@@ -5177,7 +6828,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A7)</f>
         <v/>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="20">
         <f>IFERROR(F7/30,0)</f>
         <v/>
       </c>
@@ -5208,7 +6859,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A8)</f>
         <v/>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="20">
         <f>IFERROR(F8/31,0)</f>
         <v/>
       </c>
@@ -5239,7 +6890,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A9)</f>
         <v/>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="20">
         <f>IFERROR(F9/30,0)</f>
         <v/>
       </c>
@@ -5270,7 +6921,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A10)</f>
         <v/>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="20">
         <f>IFERROR(F10/31,0)</f>
         <v/>
       </c>
@@ -5301,7 +6952,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A11)</f>
         <v/>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="20">
         <f>IFERROR(F11/31,0)</f>
         <v/>
       </c>
@@ -5332,7 +6983,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A12)</f>
         <v/>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="20">
         <f>IFERROR(F12/30,0)</f>
         <v/>
       </c>
@@ -5363,7 +7014,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A13)</f>
         <v/>
       </c>
-      <c r="G13" s="6">
+      <c r="G13" s="20">
         <f>IFERROR(F13/31,0)</f>
         <v/>
       </c>
@@ -5394,7 +7045,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A14)</f>
         <v/>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="20">
         <f>IFERROR(F14/30,0)</f>
         <v/>
       </c>
@@ -5425,7 +7076,7 @@
         <f>SUMIFS(Bookings!$F$2:$F$101,Bookings!$A$2:$A$101,A15)</f>
         <v/>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="20">
         <f>IFERROR(F15/31,0)</f>
         <v/>
       </c>
@@ -5456,12 +7107,11 @@
         <f>SUM(F4:F15)</f>
         <v/>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="21">
         <f>IFERROR(F16/365,0)</f>
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
@@ -5496,7 +7146,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A20)</f>
         <v/>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="20">
         <f>IFERROR(B20/C16,0)</f>
         <v/>
       </c>
@@ -5511,7 +7161,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A21)</f>
         <v/>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="20">
         <f>IFERROR(B21/C16,0)</f>
         <v/>
       </c>
@@ -5526,7 +7176,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A22)</f>
         <v/>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="20">
         <f>IFERROR(B22/C16,0)</f>
         <v/>
       </c>
@@ -5541,7 +7191,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A23)</f>
         <v/>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="20">
         <f>IFERROR(B23/C16,0)</f>
         <v/>
       </c>
@@ -5556,7 +7206,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A24)</f>
         <v/>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="20">
         <f>IFERROR(B24/C16,0)</f>
         <v/>
       </c>
@@ -5571,7 +7221,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A25)</f>
         <v/>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="20">
         <f>IFERROR(B25/C16,0)</f>
         <v/>
       </c>
@@ -5586,7 +7236,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A26)</f>
         <v/>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="20">
         <f>IFERROR(B26/C16,0)</f>
         <v/>
       </c>
@@ -5601,7 +7251,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A27)</f>
         <v/>
       </c>
-      <c r="C27" s="6">
+      <c r="C27" s="20">
         <f>IFERROR(B27/C16,0)</f>
         <v/>
       </c>
@@ -5616,7 +7266,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A28)</f>
         <v/>
       </c>
-      <c r="C28" s="6">
+      <c r="C28" s="20">
         <f>IFERROR(B28/C16,0)</f>
         <v/>
       </c>
@@ -5631,7 +7281,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A29)</f>
         <v/>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="20">
         <f>IFERROR(B29/C16,0)</f>
         <v/>
       </c>
@@ -5646,7 +7296,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A30)</f>
         <v/>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="20">
         <f>IFERROR(B30/C16,0)</f>
         <v/>
       </c>
@@ -5661,7 +7311,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A31)</f>
         <v/>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="20">
         <f>IFERROR(B31/C16,0)</f>
         <v/>
       </c>
@@ -5676,7 +7326,7 @@
         <f>SUMIFS(Expenses!$F$2:$F$201,Expenses!$C$2:$C$201,A32)</f>
         <v/>
       </c>
-      <c r="C32" s="6">
+      <c r="C32" s="20">
         <f>IFERROR(B32/C16,0)</f>
         <v/>
       </c>
@@ -5871,7 +7521,7 @@
           <t>% recovered</t>
         </is>
       </c>
-      <c r="B19" s="16">
+      <c r="B19" s="22">
         <f>IFERROR(B17/B6,0)</f>
         <v/>
       </c>
@@ -5893,7 +7543,7 @@
           <t>Annual occupancy rate</t>
         </is>
       </c>
-      <c r="B21" s="17">
+      <c r="B21" s="23">
         <f>'Monthly Summary'!G16</f>
         <v/>
       </c>
@@ -5945,7 +7595,7 @@
           <t>Projected years to recover investment</t>
         </is>
       </c>
-      <c r="B27" s="18">
+      <c r="B27" s="24">
         <f>IFERROR(B6/B26,0)</f>
         <v/>
       </c>
@@ -5967,9 +7617,6 @@
           <t>FUTURE EXPANSION NOTES</t>
         </is>
       </c>
-      <c r="B30" s="11" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6095,7 +7742,7 @@
         <f>B5-D5</f>
         <v/>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="20">
         <f>IFERROR(D5/B5,0)</f>
         <v/>
       </c>
@@ -6119,7 +7766,7 @@
         <f>B6-D6</f>
         <v/>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="20">
         <f>IFERROR(D6/B6,0)</f>
         <v/>
       </c>
@@ -6143,7 +7790,7 @@
         <f>B7-D7</f>
         <v/>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="20">
         <f>IFERROR(D7/B7,0)</f>
         <v/>
       </c>
@@ -6167,7 +7814,7 @@
         <f>B8-D8</f>
         <v/>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="20">
         <f>IFERROR(D8/B8,0)</f>
         <v/>
       </c>
@@ -6191,7 +7838,7 @@
         <f>B9-D9</f>
         <v/>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="20">
         <f>IFERROR(D9/B9,0)</f>
         <v/>
       </c>
@@ -6215,7 +7862,7 @@
         <f>B10-D10</f>
         <v/>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="20">
         <f>IFERROR(D10/B10,0)</f>
         <v/>
       </c>
@@ -6239,7 +7886,7 @@
         <f>B11-D11</f>
         <v/>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="20">
         <f>IFERROR(D11/B11,0)</f>
         <v/>
       </c>
@@ -6263,7 +7910,7 @@
         <f>B12-D12</f>
         <v/>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="20">
         <f>IFERROR(D12/B12,0)</f>
         <v/>
       </c>
@@ -6287,7 +7934,7 @@
         <f>B13-D13</f>
         <v/>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="20">
         <f>IFERROR(D13/B13,0)</f>
         <v/>
       </c>
@@ -6311,7 +7958,7 @@
         <f>B14-D14</f>
         <v/>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="20">
         <f>IFERROR(D14/B14,0)</f>
         <v/>
       </c>
@@ -6335,7 +7982,7 @@
         <f>B15-D15</f>
         <v/>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="20">
         <f>IFERROR(D15/B15,0)</f>
         <v/>
       </c>
@@ -6359,7 +8006,7 @@
         <f>B16-D16</f>
         <v/>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="20">
         <f>IFERROR(D16/B16,0)</f>
         <v/>
       </c>
@@ -6383,7 +8030,7 @@
         <f>B17-D17</f>
         <v/>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="20">
         <f>IFERROR(D17/B17,0)</f>
         <v/>
       </c>
@@ -6410,7 +8057,7 @@
         <f>SUM(E5:E17)</f>
         <v/>
       </c>
-      <c r="F18" s="9">
+      <c r="F18" s="21">
         <f>IFERROR(D18/B18,0)</f>
         <v/>
       </c>
@@ -6421,11 +8068,6 @@
           <t>Revenue Target</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -6478,7 +8120,7 @@
         <f>D22-B22</f>
         <v/>
       </c>
-      <c r="F22" s="6">
+      <c r="F22" s="20">
         <f>IFERROR(D22/B22,0)</f>
         <v/>
       </c>
@@ -6502,7 +8144,7 @@
         <f>D23-B23</f>
         <v/>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="20">
         <f>IFERROR(D23/B23,0)</f>
         <v/>
       </c>
@@ -6783,4 +8425,763 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>Origin</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>Round Trip Miles</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="F1" s="13" t="inlineStr">
+        <is>
+          <t>Stops/Evidence</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>IRS Rate</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
+        <is>
+          <t>Deduction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>120</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>property work, supplies</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Brookshire Brothers, McDonald’s</t>
+        </is>
+      </c>
+      <c r="G2" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H2" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>120</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>maintenance/repairs</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="G3" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H3" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>120</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>maintenance/repairs, property work, supplies</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Burger King, Brookshire Brothers, Home Depot</t>
+        </is>
+      </c>
+      <c r="G4" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H4" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="n">
+        <v>46032</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>120</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>maintenance/repairs</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="G5" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H5" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="n">
+        <v>46034</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>120</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>maintenance/repairs</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H6" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="n">
+        <v>46037</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>maintenance/repairs</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Brenco, Home Depot</t>
+        </is>
+      </c>
+      <c r="G7" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H7" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="n">
+        <v>46038</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>120</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>maintenance/repairs</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="G8" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H8" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="n">
+        <v>46039</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>120</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>supplies</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Brookshire Brothers</t>
+        </is>
+      </c>
+      <c r="G9" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H9" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="n">
+        <v>46040</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>120</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>maintenance/repairs, property work</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Ace Home Center, Pizza Hut</t>
+        </is>
+      </c>
+      <c r="G10" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H10" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="n">
+        <v>46060</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>120</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>maintenance/repairs</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Capps True Value Hardware and Ag Center</t>
+        </is>
+      </c>
+      <c r="G11" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H11" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="n">
+        <v>46063</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>120</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>maintenance/repairs, property work</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Exotic Smoke And Vape, Refund: Home Depot, Home Depot</t>
+        </is>
+      </c>
+      <c r="G12" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H12" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="25" t="n">
+        <v>46067</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>120</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>property work</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Wendy's</t>
+        </is>
+      </c>
+      <c r="G13" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H13" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="n">
+        <v>46085</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>transit fuel</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Love's Travel Stop</t>
+        </is>
+      </c>
+      <c r="G14" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H14" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="25" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>120</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>maintenance/repairs, supplies</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Ace Home Center, Brookshire Brothers</t>
+        </is>
+      </c>
+      <c r="G15" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H15" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>120</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>maintenance/repairs</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Ace Home Center</t>
+        </is>
+      </c>
+      <c r="G16" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H16" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="25" t="n">
+        <v>46100</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>120</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>property work</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>El Jimador Mexican Grill 7</t>
+        </is>
+      </c>
+      <c r="G17" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H17" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="n">
+        <v>46101</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>120</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>maintenance/repairs, transit fuel</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Gulf, Refund: Home Depot</t>
+        </is>
+      </c>
+      <c r="G18" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="25" t="n">
+        <v>46106</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>120</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>property work</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Braum's</t>
+        </is>
+      </c>
+      <c r="G19" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>120</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>maintenance/repairs, property work, transit fuel</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Taco Bell, Home Depot, Shell</t>
+        </is>
+      </c>
+      <c r="G20" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H20" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Mansfield, TX</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>360 County Road, Fairfield, TX</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>120</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>property work, supplies</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Burger King, Cooper Farms, Brookshire Brothers</t>
+        </is>
+      </c>
+      <c r="G21" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H21" s="26" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n">
+        <v>2400</v>
+      </c>
+      <c r="H22" s="27" t="n">
+        <v>1680</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update receipt column: N → CC for credit card expenses
</commit_message>
<xml_diff>
--- a/finances/kengs-landing-finance-tracker.xlsx
+++ b/finances/kengs-landing-finance-tracker.xlsx
@@ -25,12 +25,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="168" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -113,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -142,8 +141,10 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2320,7 +2321,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I5" s="2" t="n"/>
@@ -2358,7 +2359,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I6" s="2" t="n"/>
@@ -2396,7 +2397,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I7" s="2" t="n"/>
@@ -2434,7 +2435,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I8" s="2" t="n"/>
@@ -2472,7 +2473,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I9" s="2" t="n"/>
@@ -2510,7 +2511,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I10" s="2" t="n"/>
@@ -2548,7 +2549,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I11" s="2" t="n"/>
@@ -2586,7 +2587,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I12" s="2" t="n"/>
@@ -2624,7 +2625,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I13" s="2" t="n"/>
@@ -2662,7 +2663,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I14" s="2" t="n"/>
@@ -2700,7 +2701,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I15" s="2" t="n"/>
@@ -2738,7 +2739,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I16" s="2" t="n"/>
@@ -2776,7 +2777,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I17" s="2" t="n"/>
@@ -2814,7 +2815,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I18" s="2" t="n"/>
@@ -2852,7 +2853,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I19" s="2" t="n"/>
@@ -2890,7 +2891,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I20" s="2" t="n"/>
@@ -2928,7 +2929,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I21" s="2" t="n"/>
@@ -2966,7 +2967,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I22" s="2" t="n"/>
@@ -3004,7 +3005,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I23" s="2" t="n"/>
@@ -3042,7 +3043,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I24" s="2" t="n"/>
@@ -3080,7 +3081,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I25" s="2" t="n"/>
@@ -3118,7 +3119,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I26" s="2" t="n"/>
@@ -3156,7 +3157,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I27" s="2" t="n"/>
@@ -3194,7 +3195,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I28" s="2" t="n"/>
@@ -3232,7 +3233,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I29" s="2" t="n"/>
@@ -3270,7 +3271,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I30" s="2" t="n"/>
@@ -3308,7 +3309,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I31" s="2" t="n"/>
@@ -3346,7 +3347,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I32" s="2" t="n"/>
@@ -3384,7 +3385,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I33" s="2" t="n"/>
@@ -3422,7 +3423,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I34" s="2" t="n"/>
@@ -3460,7 +3461,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I35" s="2" t="n"/>
@@ -3498,7 +3499,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I36" s="2" t="n"/>
@@ -3536,7 +3537,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I37" s="2" t="n"/>
@@ -3574,7 +3575,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I38" s="2" t="n"/>
@@ -3612,7 +3613,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I39" s="2" t="n"/>
@@ -3650,7 +3651,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I40" s="2" t="n"/>
@@ -3688,7 +3689,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I41" s="2" t="n"/>
@@ -3726,7 +3727,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I42" s="2" t="n"/>
@@ -3764,7 +3765,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I43" s="2" t="n"/>
@@ -3802,7 +3803,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I44" s="2" t="n"/>
@@ -3840,7 +3841,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I45" s="2" t="n"/>
@@ -3878,7 +3879,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I46" s="2" t="n"/>
@@ -3916,7 +3917,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I47" s="2" t="n"/>
@@ -3954,7 +3955,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I48" s="2" t="n"/>
@@ -3992,7 +3993,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I49" s="2" t="n"/>
@@ -4030,7 +4031,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I50" s="2" t="n"/>
@@ -4068,7 +4069,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I51" s="2" t="n"/>
@@ -4106,7 +4107,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I52" s="2" t="n"/>
@@ -4144,7 +4145,7 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I53" s="2" t="n"/>
@@ -4182,7 +4183,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I54" s="2" t="n"/>
@@ -4220,7 +4221,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I55" s="2" t="n"/>
@@ -4258,7 +4259,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I56" s="2" t="n"/>
@@ -4296,7 +4297,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I57" s="2" t="n"/>
@@ -4334,7 +4335,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I58" s="2" t="n"/>
@@ -4372,7 +4373,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I59" s="2" t="n"/>
@@ -4410,7 +4411,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I60" s="2" t="n"/>
@@ -4448,7 +4449,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I61" s="2" t="n"/>
@@ -4486,7 +4487,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I62" s="2" t="n"/>
@@ -4524,7 +4525,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I63" s="2" t="n"/>
@@ -4562,7 +4563,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I64" s="2" t="n"/>
@@ -4600,7 +4601,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I65" s="2" t="n"/>
@@ -4638,7 +4639,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I66" s="2" t="n"/>
@@ -4676,7 +4677,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I67" s="2" t="n"/>
@@ -4714,7 +4715,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I68" s="2" t="n"/>
@@ -4752,7 +4753,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I69" s="2" t="n"/>
@@ -4790,7 +4791,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="I70" s="2" t="n"/>
@@ -8515,10 +8516,10 @@
           <t>Brookshire Brothers, McDonald’s</t>
         </is>
       </c>
-      <c r="G2" s="26" t="n">
+      <c r="G2" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H2" s="26" t="n">
+      <c r="H2" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8549,10 +8550,10 @@
           <t>Home Depot</t>
         </is>
       </c>
-      <c r="G3" s="26" t="n">
+      <c r="G3" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H3" s="26" t="n">
+      <c r="H3" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8583,10 +8584,10 @@
           <t>Burger King, Brookshire Brothers, Home Depot</t>
         </is>
       </c>
-      <c r="G4" s="26" t="n">
+      <c r="G4" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H4" s="26" t="n">
+      <c r="H4" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8617,10 +8618,10 @@
           <t>Home Depot</t>
         </is>
       </c>
-      <c r="G5" s="26" t="n">
+      <c r="G5" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H5" s="26" t="n">
+      <c r="H5" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8651,10 +8652,10 @@
           <t>Refund: Home Depot</t>
         </is>
       </c>
-      <c r="G6" s="26" t="n">
+      <c r="G6" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H6" s="26" t="n">
+      <c r="H6" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8685,10 +8686,10 @@
           <t>Brenco, Home Depot</t>
         </is>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G7" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H7" s="26" t="n">
+      <c r="H7" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8719,10 +8720,10 @@
           <t>Home Depot</t>
         </is>
       </c>
-      <c r="G8" s="26" t="n">
+      <c r="G8" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H8" s="26" t="n">
+      <c r="H8" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8753,10 +8754,10 @@
           <t>Brookshire Brothers</t>
         </is>
       </c>
-      <c r="G9" s="26" t="n">
+      <c r="G9" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H9" s="26" t="n">
+      <c r="H9" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8787,10 +8788,10 @@
           <t>Ace Home Center, Pizza Hut</t>
         </is>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H10" s="26" t="n">
+      <c r="H10" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8821,10 +8822,10 @@
           <t>Capps True Value Hardware and Ag Center</t>
         </is>
       </c>
-      <c r="G11" s="26" t="n">
+      <c r="G11" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H11" s="26" t="n">
+      <c r="H11" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8855,10 +8856,10 @@
           <t>Exotic Smoke And Vape, Refund: Home Depot, Home Depot</t>
         </is>
       </c>
-      <c r="G12" s="26" t="n">
+      <c r="G12" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H12" s="26" t="n">
+      <c r="H12" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8889,10 +8890,10 @@
           <t>Wendy's</t>
         </is>
       </c>
-      <c r="G13" s="26" t="n">
+      <c r="G13" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H13" s="26" t="n">
+      <c r="H13" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8923,10 +8924,10 @@
           <t>Love's Travel Stop</t>
         </is>
       </c>
-      <c r="G14" s="26" t="n">
+      <c r="G14" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H14" s="26" t="n">
+      <c r="H14" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8957,10 +8958,10 @@
           <t>Ace Home Center, Brookshire Brothers</t>
         </is>
       </c>
-      <c r="G15" s="26" t="n">
+      <c r="G15" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H15" s="26" t="n">
+      <c r="H15" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -8991,10 +8992,10 @@
           <t>Ace Home Center</t>
         </is>
       </c>
-      <c r="G16" s="26" t="n">
+      <c r="G16" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H16" s="26" t="n">
+      <c r="H16" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -9025,10 +9026,10 @@
           <t>El Jimador Mexican Grill 7</t>
         </is>
       </c>
-      <c r="G17" s="26" t="n">
+      <c r="G17" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H17" s="26" t="n">
+      <c r="H17" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -9059,10 +9060,10 @@
           <t>Gulf, Refund: Home Depot</t>
         </is>
       </c>
-      <c r="G18" s="26" t="n">
+      <c r="G18" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H18" s="26" t="n">
+      <c r="H18" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -9093,10 +9094,10 @@
           <t>Braum's</t>
         </is>
       </c>
-      <c r="G19" s="26" t="n">
+      <c r="G19" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H19" s="26" t="n">
+      <c r="H19" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -9127,10 +9128,10 @@
           <t>Taco Bell, Home Depot, Shell</t>
         </is>
       </c>
-      <c r="G20" s="26" t="n">
+      <c r="G20" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H20" s="26" t="n">
+      <c r="H20" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -9161,10 +9162,10 @@
           <t>Burger King, Cooper Farms, Brookshire Brothers</t>
         </is>
       </c>
-      <c r="G21" s="26" t="n">
+      <c r="G21" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="H21" s="26" t="n">
+      <c r="H21" s="28" t="n">
         <v>84</v>
       </c>
     </row>
@@ -9177,7 +9178,7 @@
       <c r="D22" s="13" t="n">
         <v>2400</v>
       </c>
-      <c r="H22" s="27" t="n">
+      <c r="H22" s="29" t="n">
         <v>1680</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dynamic improvements: compute from expenses, not hardcoded estimate
- Removed hardcoded $10K improvements guess from Investment & ROI
- Dashboard now computes improvements from actual Business-status expenses
- Split $7K cash withdrawal into documented components:
  - Jeff Yancey cash $1,200 (Business, text msg evidence)
  - ATM $500 probable Jeff payment (Review)
  - Golf carts $2,400 (Review — pending bill of sale)
  - Unaccounted $3,400 (Review — do NOT report until documented)
- Budget tab ROI sidebar shows documented vs pending amounts
- Overview KPI shows actual total investment with improvement breakdown
</commit_message>
<xml_diff>
--- a/finances/kengs-landing-finance-tracker.xlsx
+++ b/finances/kengs-landing-finance-tracker.xlsx
@@ -66,7 +66,7 @@
       <color rgb="00666666"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +89,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0B2"/>
+        <bgColor rgb="00FFE0B2"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -157,6 +163,9 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7177,45 +7186,45 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="31" t="n">
+      <c r="A119" s="3" t="n">
         <v>45985</v>
       </c>
-      <c r="B119" s="32" t="inlineStr">
+      <c r="B119" s="2" t="inlineStr">
         <is>
           <t>November 2025</t>
         </is>
       </c>
-      <c r="C119" s="32" t="inlineStr">
+      <c r="C119" s="2" t="inlineStr">
         <is>
           <t>Repairs &amp; maintenance</t>
         </is>
       </c>
-      <c r="D119" s="32" t="inlineStr">
-        <is>
-          <t>Cash withdrawal</t>
-        </is>
-      </c>
-      <c r="E119" s="32" t="inlineStr">
-        <is>
-          <t>Cash for Jeff Yancey + skid steer for 360 CR land clearing — need to determine split</t>
-        </is>
-      </c>
-      <c r="F119" s="33" t="n">
-        <v>7000</v>
-      </c>
-      <c r="G119" s="32" t="inlineStr">
-        <is>
-          <t>Cash (3125)</t>
-        </is>
-      </c>
-      <c r="H119" s="32" t="inlineStr">
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>Jeff Yancey (cash)</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>Cash payment for contractor work — text messages as evidence</t>
+        </is>
+      </c>
+      <c r="F119" s="4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I119" s="32" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>Business</t>
         </is>
       </c>
     </row>
@@ -7235,12 +7244,12 @@
       </c>
       <c r="D120" s="32" t="inlineStr">
         <is>
-          <t>ATM Cash</t>
+          <t>Jeff Yancey (cash probable)</t>
         </is>
       </c>
       <c r="E120" s="32" t="inlineStr">
         <is>
-          <t>Cash — probably Jeff Yancey payment</t>
+          <t>ATM cash — probably Jeff Yancey payment, text msg evidence</t>
         </is>
       </c>
       <c r="F120" s="33" t="n">
@@ -7248,7 +7257,7 @@
       </c>
       <c r="G120" s="32" t="inlineStr">
         <is>
-          <t>Cash (3125)</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="H120" s="32" t="inlineStr">
@@ -7865,32 +7874,90 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="3" t="n"/>
-      <c r="B135" s="2">
-        <f>IF(A135="","",TEXT(A135,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C135" s="2" t="n"/>
-      <c r="D135" s="2" t="n"/>
-      <c r="E135" s="2" t="n"/>
-      <c r="F135" s="4" t="n"/>
-      <c r="G135" s="2" t="n"/>
-      <c r="H135" s="2" t="n"/>
-      <c r="I135" s="2" t="n"/>
+      <c r="A135" s="34" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B135" s="35" t="inlineStr">
+        <is>
+          <t>November 2025</t>
+        </is>
+      </c>
+      <c r="C135" s="35" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="D135" s="35" t="inlineStr">
+        <is>
+          <t>Golf Carts (2x)</t>
+        </is>
+      </c>
+      <c r="E135" s="35" t="inlineStr">
+        <is>
+          <t>Two golf carts for STR property — PENDING: need bill of sale to deduct</t>
+        </is>
+      </c>
+      <c r="F135" s="36" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G135" s="35" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="H135" s="35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I135" s="35" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
     </row>
     <row r="136">
-      <c r="A136" s="3" t="n"/>
-      <c r="B136" s="2">
-        <f>IF(A136="","",TEXT(A136,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C136" s="2" t="n"/>
-      <c r="D136" s="2" t="n"/>
-      <c r="E136" s="2" t="n"/>
-      <c r="F136" s="4" t="n"/>
-      <c r="G136" s="2" t="n"/>
-      <c r="H136" s="2" t="n"/>
-      <c r="I136" s="2" t="n"/>
+      <c r="A136" s="34" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B136" s="35" t="inlineStr">
+        <is>
+          <t>November 2025</t>
+        </is>
+      </c>
+      <c r="C136" s="35" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D136" s="35" t="inlineStr">
+        <is>
+          <t>Unaccounted Cash</t>
+        </is>
+      </c>
+      <c r="E136" s="35" t="inlineStr">
+        <is>
+          <t>Remaining from $7,500 cash withdrawal — INVESTIGATE: $1,200 Jeff + $2,400 carts + $500 ATM = $4,100 accounted. This $3,400 is unaccounted. Do NOT report until documented.</t>
+        </is>
+      </c>
+      <c r="F136" s="36" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G136" s="35" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="H136" s="35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I136" s="35" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="n"/>
@@ -9549,6 +9616,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -9574,7 +9642,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Normalize expense category casing (56 entries)
</commit_message>
<xml_diff>
--- a/finances/kengs-landing-finance-tracker.xlsx
+++ b/finances/kengs-landing-finance-tracker.xlsx
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Cleaning &amp; Turnover</t>
+          <t>Cleaning &amp; turnover</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Cleaning &amp; Turnover</t>
+          <t>Cleaning &amp; turnover</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Cleaning &amp; Turnover</t>
+          <t>Cleaning &amp; turnover</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="C9" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D9" s="32" t="inlineStr">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="C10" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D10" s="32" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="C13" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D13" s="32" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D21" s="32" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="C22" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D22" s="32" t="inlineStr">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="C29" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D29" s="32" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="C30" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D30" s="32" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="C31" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D31" s="32" t="inlineStr">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="C32" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D32" s="32" t="inlineStr">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="C34" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D34" s="32" t="inlineStr">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="C35" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D35" s="32" t="inlineStr">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="C37" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D37" s="32" t="inlineStr">
@@ -3745,7 +3745,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="C43" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D43" s="32" t="inlineStr">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="C44" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D44" s="32" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C45" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D45" s="32" t="inlineStr">
@@ -4123,7 +4123,7 @@
       </c>
       <c r="C47" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D47" s="32" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="C48" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D48" s="32" t="inlineStr">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="C49" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D49" s="32" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -4375,7 +4375,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -4459,7 +4459,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -4585,7 +4585,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -4711,7 +4711,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -4753,7 +4753,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Professional Services</t>
+          <t>Professional services</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -4795,7 +4795,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -4837,7 +4837,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Travel / Mileage</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -5089,7 +5089,7 @@
       </c>
       <c r="C70" s="32" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>Repairs &amp; maintenance</t>
         </is>
       </c>
       <c r="D70" s="32" t="inlineStr">
@@ -9616,7 +9616,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix dashboard bugs, add Tax Period column, export audit trail
Dashboard fixes:
- Normalize CATEGORIES constant to match Excel casing (Repairs & maintenance, etc.)
- Add case-insensitive category matching in ytdExpenseByCategory()
- Fix localStorage migration: normalize status, category, and tax period on load
- Fix Investment Recovery KPI: show revenue-based recovery instead of misleading 0%
- ROI section: show revenue recovered, net profit, projected payback

Tax Period:
- Add Tax Period column to Excel (Pre-Service vs Operational, cutoff: 2026-03-01)
- Dashboard reads/writes/displays Tax Period with color-coded badges
- Expense table footer shows Pre-Service vs Operational totals
- Overview KPI card shows pre-service expense breakdown
- Date changes auto-recompute tax period

Audit trail:
- Export all 135 expenses as CSV to finances/2026/expenses/
- Clean up 65 empty trailing rows in Excel
</commit_message>
<xml_diff>
--- a/finances/kengs-landing-finance-tracker.xlsx
+++ b/finances/kengs-landing-finance-tracker.xlsx
@@ -2162,7 +2162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I201"/>
+  <dimension ref="A1:J136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -2222,6 +2222,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Tax Period</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -2264,6 +2269,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -2306,6 +2316,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -2348,6 +2363,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -2390,6 +2410,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -2432,6 +2457,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -2474,6 +2504,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -2516,6 +2551,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="31" t="n">
@@ -2558,6 +2598,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="31" t="n">
@@ -2600,6 +2645,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -2642,6 +2692,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -2684,6 +2739,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="31" t="n">
@@ -2726,6 +2786,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -2768,6 +2833,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -2810,6 +2880,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -2852,6 +2927,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -2894,6 +2974,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -2936,6 +3021,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -2978,6 +3068,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -3020,6 +3115,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="31" t="n">
@@ -3062,6 +3162,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="31" t="n">
@@ -3104,6 +3209,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -3146,6 +3256,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -3188,6 +3303,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -3230,6 +3350,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -3272,6 +3397,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -3314,6 +3444,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -3356,6 +3491,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="31" t="n">
@@ -3398,6 +3538,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="31" t="n">
@@ -3440,6 +3585,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="31" t="n">
@@ -3482,6 +3632,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="31" t="n">
@@ -3524,6 +3679,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -3566,6 +3726,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="31" t="n">
@@ -3608,6 +3773,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="31" t="n">
@@ -3650,6 +3820,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -3692,6 +3867,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="31" t="n">
@@ -3734,6 +3914,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -3776,6 +3961,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -3818,6 +4008,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -3860,6 +4055,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -3902,6 +4102,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -3944,6 +4149,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="31" t="n">
@@ -3986,6 +4196,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="31" t="n">
@@ -4028,6 +4243,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="31" t="n">
@@ -4070,6 +4290,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -4112,6 +4337,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="31" t="n">
@@ -4154,6 +4384,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="31" t="n">
@@ -4196,6 +4431,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="31" t="n">
@@ -4238,6 +4478,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
@@ -4280,6 +4525,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -4322,6 +4572,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -4364,6 +4619,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
@@ -4406,6 +4666,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -4448,6 +4713,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
@@ -4490,6 +4760,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n">
@@ -4532,6 +4807,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -4574,6 +4854,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -4616,6 +4901,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -4658,6 +4948,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
@@ -4700,6 +4995,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
@@ -4742,6 +5042,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n">
@@ -4784,6 +5089,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -4826,6 +5136,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n">
@@ -4868,6 +5183,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -4910,6 +5230,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n">
@@ -4952,6 +5277,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -4994,6 +5324,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
@@ -5036,6 +5371,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
@@ -5078,6 +5418,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="31" t="n">
@@ -5120,6 +5465,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n">
@@ -5163,6 +5513,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -5206,6 +5561,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
@@ -5249,6 +5609,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -5292,6 +5657,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
@@ -5335,6 +5705,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
@@ -5378,6 +5753,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
@@ -5421,6 +5801,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
@@ -5464,6 +5849,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
@@ -5507,6 +5897,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
@@ -5550,6 +5945,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
@@ -5593,6 +5993,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n">
@@ -5636,6 +6041,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n">
@@ -5679,6 +6089,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n">
@@ -5722,6 +6137,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
@@ -5765,6 +6185,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n">
@@ -5808,6 +6233,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n">
@@ -5851,6 +6281,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n">
@@ -5894,6 +6329,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n">
@@ -5937,6 +6377,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n">
@@ -5980,6 +6425,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n">
@@ -6023,6 +6473,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="31" t="n">
@@ -6066,6 +6521,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="31" t="n">
@@ -6109,6 +6569,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n">
@@ -6152,6 +6617,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
@@ -6195,6 +6665,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n">
@@ -6238,6 +6713,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n">
@@ -6281,6 +6761,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n">
@@ -6324,6 +6809,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n">
@@ -6367,6 +6857,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n">
@@ -6410,6 +6905,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n">
@@ -6453,6 +6953,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n">
@@ -6496,6 +7001,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n">
@@ -6539,6 +7049,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n">
@@ -6582,6 +7097,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n">
@@ -6625,6 +7145,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n">
@@ -6668,6 +7193,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n">
@@ -6711,6 +7241,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n">
@@ -6754,6 +7289,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n">
@@ -6797,6 +7337,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n">
@@ -6840,6 +7385,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="n">
@@ -6883,6 +7433,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="31" t="n">
@@ -6926,6 +7481,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="31" t="n">
@@ -6969,6 +7529,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="31" t="n">
@@ -7012,6 +7577,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="31" t="n">
@@ -7055,6 +7625,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="31" t="n">
@@ -7098,6 +7673,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="n">
@@ -7141,6 +7721,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="n">
@@ -7184,6 +7769,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="n">
@@ -7227,6 +7817,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="31" t="n">
@@ -7270,6 +7865,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="n">
@@ -7313,6 +7913,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="n">
@@ -7356,6 +7961,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="n">
@@ -7399,6 +8009,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="n">
@@ -7442,6 +8057,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="n">
@@ -7485,6 +8105,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="n">
@@ -7528,6 +8153,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="n">
@@ -7571,6 +8201,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="n">
@@ -7614,6 +8249,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="n">
@@ -7657,6 +8297,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="n">
@@ -7700,6 +8345,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="n">
@@ -7743,6 +8393,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="n">
@@ -7786,6 +8441,11 @@
           <t>Business</t>
         </is>
       </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="31" t="n">
@@ -7829,6 +8489,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="31" t="n">
@@ -7872,6 +8537,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="34" t="n">
@@ -7915,6 +8585,11 @@
           <t>Review</t>
         </is>
       </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="34" t="n">
@@ -7958,916 +8633,11 @@
           <t>Review</t>
         </is>
       </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="3" t="n"/>
-      <c r="B137" s="2">
-        <f>IF(A137="","",TEXT(A137,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C137" s="2" t="n"/>
-      <c r="D137" s="2" t="n"/>
-      <c r="E137" s="2" t="n"/>
-      <c r="F137" s="4" t="n"/>
-      <c r="G137" s="2" t="n"/>
-      <c r="H137" s="2" t="n"/>
-      <c r="I137" s="2" t="n"/>
-    </row>
-    <row r="138">
-      <c r="A138" s="3" t="n"/>
-      <c r="B138" s="2">
-        <f>IF(A138="","",TEXT(A138,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C138" s="2" t="n"/>
-      <c r="D138" s="2" t="n"/>
-      <c r="E138" s="2" t="n"/>
-      <c r="F138" s="4" t="n"/>
-      <c r="G138" s="2" t="n"/>
-      <c r="H138" s="2" t="n"/>
-      <c r="I138" s="2" t="n"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="3" t="n"/>
-      <c r="B139" s="2">
-        <f>IF(A139="","",TEXT(A139,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C139" s="2" t="n"/>
-      <c r="D139" s="2" t="n"/>
-      <c r="E139" s="2" t="n"/>
-      <c r="F139" s="4" t="n"/>
-      <c r="G139" s="2" t="n"/>
-      <c r="H139" s="2" t="n"/>
-      <c r="I139" s="2" t="n"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="3" t="n"/>
-      <c r="B140" s="2">
-        <f>IF(A140="","",TEXT(A140,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C140" s="2" t="n"/>
-      <c r="D140" s="2" t="n"/>
-      <c r="E140" s="2" t="n"/>
-      <c r="F140" s="4" t="n"/>
-      <c r="G140" s="2" t="n"/>
-      <c r="H140" s="2" t="n"/>
-      <c r="I140" s="2" t="n"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="3" t="n"/>
-      <c r="B141" s="2">
-        <f>IF(A141="","",TEXT(A141,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C141" s="2" t="n"/>
-      <c r="D141" s="2" t="n"/>
-      <c r="E141" s="2" t="n"/>
-      <c r="F141" s="4" t="n"/>
-      <c r="G141" s="2" t="n"/>
-      <c r="H141" s="2" t="n"/>
-      <c r="I141" s="2" t="n"/>
-    </row>
-    <row r="142">
-      <c r="A142" s="3" t="n"/>
-      <c r="B142" s="2">
-        <f>IF(A142="","",TEXT(A142,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C142" s="2" t="n"/>
-      <c r="D142" s="2" t="n"/>
-      <c r="E142" s="2" t="n"/>
-      <c r="F142" s="4" t="n"/>
-      <c r="G142" s="2" t="n"/>
-      <c r="H142" s="2" t="n"/>
-      <c r="I142" s="2" t="n"/>
-    </row>
-    <row r="143">
-      <c r="A143" s="3" t="n"/>
-      <c r="B143" s="2">
-        <f>IF(A143="","",TEXT(A143,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C143" s="2" t="n"/>
-      <c r="D143" s="2" t="n"/>
-      <c r="E143" s="2" t="n"/>
-      <c r="F143" s="4" t="n"/>
-      <c r="G143" s="2" t="n"/>
-      <c r="H143" s="2" t="n"/>
-      <c r="I143" s="2" t="n"/>
-    </row>
-    <row r="144">
-      <c r="A144" s="3" t="n"/>
-      <c r="B144" s="2">
-        <f>IF(A144="","",TEXT(A144,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C144" s="2" t="n"/>
-      <c r="D144" s="2" t="n"/>
-      <c r="E144" s="2" t="n"/>
-      <c r="F144" s="4" t="n"/>
-      <c r="G144" s="2" t="n"/>
-      <c r="H144" s="2" t="n"/>
-      <c r="I144" s="2" t="n"/>
-    </row>
-    <row r="145">
-      <c r="A145" s="3" t="n"/>
-      <c r="B145" s="2">
-        <f>IF(A145="","",TEXT(A145,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C145" s="2" t="n"/>
-      <c r="D145" s="2" t="n"/>
-      <c r="E145" s="2" t="n"/>
-      <c r="F145" s="4" t="n"/>
-      <c r="G145" s="2" t="n"/>
-      <c r="H145" s="2" t="n"/>
-      <c r="I145" s="2" t="n"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="3" t="n"/>
-      <c r="B146" s="2">
-        <f>IF(A146="","",TEXT(A146,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C146" s="2" t="n"/>
-      <c r="D146" s="2" t="n"/>
-      <c r="E146" s="2" t="n"/>
-      <c r="F146" s="4" t="n"/>
-      <c r="G146" s="2" t="n"/>
-      <c r="H146" s="2" t="n"/>
-      <c r="I146" s="2" t="n"/>
-    </row>
-    <row r="147">
-      <c r="A147" s="3" t="n"/>
-      <c r="B147" s="2">
-        <f>IF(A147="","",TEXT(A147,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C147" s="2" t="n"/>
-      <c r="D147" s="2" t="n"/>
-      <c r="E147" s="2" t="n"/>
-      <c r="F147" s="4" t="n"/>
-      <c r="G147" s="2" t="n"/>
-      <c r="H147" s="2" t="n"/>
-      <c r="I147" s="2" t="n"/>
-    </row>
-    <row r="148">
-      <c r="A148" s="3" t="n"/>
-      <c r="B148" s="2">
-        <f>IF(A148="","",TEXT(A148,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C148" s="2" t="n"/>
-      <c r="D148" s="2" t="n"/>
-      <c r="E148" s="2" t="n"/>
-      <c r="F148" s="4" t="n"/>
-      <c r="G148" s="2" t="n"/>
-      <c r="H148" s="2" t="n"/>
-      <c r="I148" s="2" t="n"/>
-    </row>
-    <row r="149">
-      <c r="A149" s="3" t="n"/>
-      <c r="B149" s="2">
-        <f>IF(A149="","",TEXT(A149,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C149" s="2" t="n"/>
-      <c r="D149" s="2" t="n"/>
-      <c r="E149" s="2" t="n"/>
-      <c r="F149" s="4" t="n"/>
-      <c r="G149" s="2" t="n"/>
-      <c r="H149" s="2" t="n"/>
-      <c r="I149" s="2" t="n"/>
-    </row>
-    <row r="150">
-      <c r="A150" s="3" t="n"/>
-      <c r="B150" s="2">
-        <f>IF(A150="","",TEXT(A150,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C150" s="2" t="n"/>
-      <c r="D150" s="2" t="n"/>
-      <c r="E150" s="2" t="n"/>
-      <c r="F150" s="4" t="n"/>
-      <c r="G150" s="2" t="n"/>
-      <c r="H150" s="2" t="n"/>
-      <c r="I150" s="2" t="n"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="3" t="n"/>
-      <c r="B151" s="2">
-        <f>IF(A151="","",TEXT(A151,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C151" s="2" t="n"/>
-      <c r="D151" s="2" t="n"/>
-      <c r="E151" s="2" t="n"/>
-      <c r="F151" s="4" t="n"/>
-      <c r="G151" s="2" t="n"/>
-      <c r="H151" s="2" t="n"/>
-      <c r="I151" s="2" t="n"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="3" t="n"/>
-      <c r="B152" s="2">
-        <f>IF(A152="","",TEXT(A152,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C152" s="2" t="n"/>
-      <c r="D152" s="2" t="n"/>
-      <c r="E152" s="2" t="n"/>
-      <c r="F152" s="4" t="n"/>
-      <c r="G152" s="2" t="n"/>
-      <c r="H152" s="2" t="n"/>
-      <c r="I152" s="2" t="n"/>
-    </row>
-    <row r="153">
-      <c r="A153" s="3" t="n"/>
-      <c r="B153" s="2">
-        <f>IF(A153="","",TEXT(A153,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C153" s="2" t="n"/>
-      <c r="D153" s="2" t="n"/>
-      <c r="E153" s="2" t="n"/>
-      <c r="F153" s="4" t="n"/>
-      <c r="G153" s="2" t="n"/>
-      <c r="H153" s="2" t="n"/>
-      <c r="I153" s="2" t="n"/>
-    </row>
-    <row r="154">
-      <c r="A154" s="3" t="n"/>
-      <c r="B154" s="2">
-        <f>IF(A154="","",TEXT(A154,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C154" s="2" t="n"/>
-      <c r="D154" s="2" t="n"/>
-      <c r="E154" s="2" t="n"/>
-      <c r="F154" s="4" t="n"/>
-      <c r="G154" s="2" t="n"/>
-      <c r="H154" s="2" t="n"/>
-      <c r="I154" s="2" t="n"/>
-    </row>
-    <row r="155">
-      <c r="A155" s="3" t="n"/>
-      <c r="B155" s="2">
-        <f>IF(A155="","",TEXT(A155,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C155" s="2" t="n"/>
-      <c r="D155" s="2" t="n"/>
-      <c r="E155" s="2" t="n"/>
-      <c r="F155" s="4" t="n"/>
-      <c r="G155" s="2" t="n"/>
-      <c r="H155" s="2" t="n"/>
-      <c r="I155" s="2" t="n"/>
-    </row>
-    <row r="156">
-      <c r="A156" s="3" t="n"/>
-      <c r="B156" s="2">
-        <f>IF(A156="","",TEXT(A156,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C156" s="2" t="n"/>
-      <c r="D156" s="2" t="n"/>
-      <c r="E156" s="2" t="n"/>
-      <c r="F156" s="4" t="n"/>
-      <c r="G156" s="2" t="n"/>
-      <c r="H156" s="2" t="n"/>
-      <c r="I156" s="2" t="n"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="3" t="n"/>
-      <c r="B157" s="2">
-        <f>IF(A157="","",TEXT(A157,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C157" s="2" t="n"/>
-      <c r="D157" s="2" t="n"/>
-      <c r="E157" s="2" t="n"/>
-      <c r="F157" s="4" t="n"/>
-      <c r="G157" s="2" t="n"/>
-      <c r="H157" s="2" t="n"/>
-      <c r="I157" s="2" t="n"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="3" t="n"/>
-      <c r="B158" s="2">
-        <f>IF(A158="","",TEXT(A158,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C158" s="2" t="n"/>
-      <c r="D158" s="2" t="n"/>
-      <c r="E158" s="2" t="n"/>
-      <c r="F158" s="4" t="n"/>
-      <c r="G158" s="2" t="n"/>
-      <c r="H158" s="2" t="n"/>
-      <c r="I158" s="2" t="n"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="3" t="n"/>
-      <c r="B159" s="2">
-        <f>IF(A159="","",TEXT(A159,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C159" s="2" t="n"/>
-      <c r="D159" s="2" t="n"/>
-      <c r="E159" s="2" t="n"/>
-      <c r="F159" s="4" t="n"/>
-      <c r="G159" s="2" t="n"/>
-      <c r="H159" s="2" t="n"/>
-      <c r="I159" s="2" t="n"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="3" t="n"/>
-      <c r="B160" s="2">
-        <f>IF(A160="","",TEXT(A160,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C160" s="2" t="n"/>
-      <c r="D160" s="2" t="n"/>
-      <c r="E160" s="2" t="n"/>
-      <c r="F160" s="4" t="n"/>
-      <c r="G160" s="2" t="n"/>
-      <c r="H160" s="2" t="n"/>
-      <c r="I160" s="2" t="n"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="3" t="n"/>
-      <c r="B161" s="2">
-        <f>IF(A161="","",TEXT(A161,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C161" s="2" t="n"/>
-      <c r="D161" s="2" t="n"/>
-      <c r="E161" s="2" t="n"/>
-      <c r="F161" s="4" t="n"/>
-      <c r="G161" s="2" t="n"/>
-      <c r="H161" s="2" t="n"/>
-      <c r="I161" s="2" t="n"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="3" t="n"/>
-      <c r="B162" s="2">
-        <f>IF(A162="","",TEXT(A162,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C162" s="2" t="n"/>
-      <c r="D162" s="2" t="n"/>
-      <c r="E162" s="2" t="n"/>
-      <c r="F162" s="4" t="n"/>
-      <c r="G162" s="2" t="n"/>
-      <c r="H162" s="2" t="n"/>
-      <c r="I162" s="2" t="n"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="3" t="n"/>
-      <c r="B163" s="2">
-        <f>IF(A163="","",TEXT(A163,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C163" s="2" t="n"/>
-      <c r="D163" s="2" t="n"/>
-      <c r="E163" s="2" t="n"/>
-      <c r="F163" s="4" t="n"/>
-      <c r="G163" s="2" t="n"/>
-      <c r="H163" s="2" t="n"/>
-      <c r="I163" s="2" t="n"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="3" t="n"/>
-      <c r="B164" s="2">
-        <f>IF(A164="","",TEXT(A164,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C164" s="2" t="n"/>
-      <c r="D164" s="2" t="n"/>
-      <c r="E164" s="2" t="n"/>
-      <c r="F164" s="4" t="n"/>
-      <c r="G164" s="2" t="n"/>
-      <c r="H164" s="2" t="n"/>
-      <c r="I164" s="2" t="n"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="3" t="n"/>
-      <c r="B165" s="2">
-        <f>IF(A165="","",TEXT(A165,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C165" s="2" t="n"/>
-      <c r="D165" s="2" t="n"/>
-      <c r="E165" s="2" t="n"/>
-      <c r="F165" s="4" t="n"/>
-      <c r="G165" s="2" t="n"/>
-      <c r="H165" s="2" t="n"/>
-      <c r="I165" s="2" t="n"/>
-    </row>
-    <row r="166">
-      <c r="A166" s="3" t="n"/>
-      <c r="B166" s="2">
-        <f>IF(A166="","",TEXT(A166,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C166" s="2" t="n"/>
-      <c r="D166" s="2" t="n"/>
-      <c r="E166" s="2" t="n"/>
-      <c r="F166" s="4" t="n"/>
-      <c r="G166" s="2" t="n"/>
-      <c r="H166" s="2" t="n"/>
-      <c r="I166" s="2" t="n"/>
-    </row>
-    <row r="167">
-      <c r="A167" s="3" t="n"/>
-      <c r="B167" s="2">
-        <f>IF(A167="","",TEXT(A167,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C167" s="2" t="n"/>
-      <c r="D167" s="2" t="n"/>
-      <c r="E167" s="2" t="n"/>
-      <c r="F167" s="4" t="n"/>
-      <c r="G167" s="2" t="n"/>
-      <c r="H167" s="2" t="n"/>
-      <c r="I167" s="2" t="n"/>
-    </row>
-    <row r="168">
-      <c r="A168" s="3" t="n"/>
-      <c r="B168" s="2">
-        <f>IF(A168="","",TEXT(A168,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C168" s="2" t="n"/>
-      <c r="D168" s="2" t="n"/>
-      <c r="E168" s="2" t="n"/>
-      <c r="F168" s="4" t="n"/>
-      <c r="G168" s="2" t="n"/>
-      <c r="H168" s="2" t="n"/>
-      <c r="I168" s="2" t="n"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="3" t="n"/>
-      <c r="B169" s="2">
-        <f>IF(A169="","",TEXT(A169,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C169" s="2" t="n"/>
-      <c r="D169" s="2" t="n"/>
-      <c r="E169" s="2" t="n"/>
-      <c r="F169" s="4" t="n"/>
-      <c r="G169" s="2" t="n"/>
-      <c r="H169" s="2" t="n"/>
-      <c r="I169" s="2" t="n"/>
-    </row>
-    <row r="170">
-      <c r="A170" s="3" t="n"/>
-      <c r="B170" s="2">
-        <f>IF(A170="","",TEXT(A170,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C170" s="2" t="n"/>
-      <c r="D170" s="2" t="n"/>
-      <c r="E170" s="2" t="n"/>
-      <c r="F170" s="4" t="n"/>
-      <c r="G170" s="2" t="n"/>
-      <c r="H170" s="2" t="n"/>
-      <c r="I170" s="2" t="n"/>
-    </row>
-    <row r="171">
-      <c r="A171" s="3" t="n"/>
-      <c r="B171" s="2">
-        <f>IF(A171="","",TEXT(A171,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C171" s="2" t="n"/>
-      <c r="D171" s="2" t="n"/>
-      <c r="E171" s="2" t="n"/>
-      <c r="F171" s="4" t="n"/>
-      <c r="G171" s="2" t="n"/>
-      <c r="H171" s="2" t="n"/>
-      <c r="I171" s="2" t="n"/>
-    </row>
-    <row r="172">
-      <c r="A172" s="3" t="n"/>
-      <c r="B172" s="2">
-        <f>IF(A172="","",TEXT(A172,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C172" s="2" t="n"/>
-      <c r="D172" s="2" t="n"/>
-      <c r="E172" s="2" t="n"/>
-      <c r="F172" s="4" t="n"/>
-      <c r="G172" s="2" t="n"/>
-      <c r="H172" s="2" t="n"/>
-      <c r="I172" s="2" t="n"/>
-    </row>
-    <row r="173">
-      <c r="A173" s="3" t="n"/>
-      <c r="B173" s="2">
-        <f>IF(A173="","",TEXT(A173,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C173" s="2" t="n"/>
-      <c r="D173" s="2" t="n"/>
-      <c r="E173" s="2" t="n"/>
-      <c r="F173" s="4" t="n"/>
-      <c r="G173" s="2" t="n"/>
-      <c r="H173" s="2" t="n"/>
-      <c r="I173" s="2" t="n"/>
-    </row>
-    <row r="174">
-      <c r="A174" s="3" t="n"/>
-      <c r="B174" s="2">
-        <f>IF(A174="","",TEXT(A174,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C174" s="2" t="n"/>
-      <c r="D174" s="2" t="n"/>
-      <c r="E174" s="2" t="n"/>
-      <c r="F174" s="4" t="n"/>
-      <c r="G174" s="2" t="n"/>
-      <c r="H174" s="2" t="n"/>
-      <c r="I174" s="2" t="n"/>
-    </row>
-    <row r="175">
-      <c r="A175" s="3" t="n"/>
-      <c r="B175" s="2">
-        <f>IF(A175="","",TEXT(A175,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C175" s="2" t="n"/>
-      <c r="D175" s="2" t="n"/>
-      <c r="E175" s="2" t="n"/>
-      <c r="F175" s="4" t="n"/>
-      <c r="G175" s="2" t="n"/>
-      <c r="H175" s="2" t="n"/>
-      <c r="I175" s="2" t="n"/>
-    </row>
-    <row r="176">
-      <c r="A176" s="3" t="n"/>
-      <c r="B176" s="2">
-        <f>IF(A176="","",TEXT(A176,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C176" s="2" t="n"/>
-      <c r="D176" s="2" t="n"/>
-      <c r="E176" s="2" t="n"/>
-      <c r="F176" s="4" t="n"/>
-      <c r="G176" s="2" t="n"/>
-      <c r="H176" s="2" t="n"/>
-      <c r="I176" s="2" t="n"/>
-    </row>
-    <row r="177">
-      <c r="A177" s="3" t="n"/>
-      <c r="B177" s="2">
-        <f>IF(A177="","",TEXT(A177,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C177" s="2" t="n"/>
-      <c r="D177" s="2" t="n"/>
-      <c r="E177" s="2" t="n"/>
-      <c r="F177" s="4" t="n"/>
-      <c r="G177" s="2" t="n"/>
-      <c r="H177" s="2" t="n"/>
-      <c r="I177" s="2" t="n"/>
-    </row>
-    <row r="178">
-      <c r="A178" s="3" t="n"/>
-      <c r="B178" s="2">
-        <f>IF(A178="","",TEXT(A178,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C178" s="2" t="n"/>
-      <c r="D178" s="2" t="n"/>
-      <c r="E178" s="2" t="n"/>
-      <c r="F178" s="4" t="n"/>
-      <c r="G178" s="2" t="n"/>
-      <c r="H178" s="2" t="n"/>
-      <c r="I178" s="2" t="n"/>
-    </row>
-    <row r="179">
-      <c r="A179" s="3" t="n"/>
-      <c r="B179" s="2">
-        <f>IF(A179="","",TEXT(A179,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C179" s="2" t="n"/>
-      <c r="D179" s="2" t="n"/>
-      <c r="E179" s="2" t="n"/>
-      <c r="F179" s="4" t="n"/>
-      <c r="G179" s="2" t="n"/>
-      <c r="H179" s="2" t="n"/>
-      <c r="I179" s="2" t="n"/>
-    </row>
-    <row r="180">
-      <c r="A180" s="3" t="n"/>
-      <c r="B180" s="2">
-        <f>IF(A180="","",TEXT(A180,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C180" s="2" t="n"/>
-      <c r="D180" s="2" t="n"/>
-      <c r="E180" s="2" t="n"/>
-      <c r="F180" s="4" t="n"/>
-      <c r="G180" s="2" t="n"/>
-      <c r="H180" s="2" t="n"/>
-      <c r="I180" s="2" t="n"/>
-    </row>
-    <row r="181">
-      <c r="A181" s="3" t="n"/>
-      <c r="B181" s="2">
-        <f>IF(A181="","",TEXT(A181,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C181" s="2" t="n"/>
-      <c r="D181" s="2" t="n"/>
-      <c r="E181" s="2" t="n"/>
-      <c r="F181" s="4" t="n"/>
-      <c r="G181" s="2" t="n"/>
-      <c r="H181" s="2" t="n"/>
-      <c r="I181" s="2" t="n"/>
-    </row>
-    <row r="182">
-      <c r="A182" s="3" t="n"/>
-      <c r="B182" s="2">
-        <f>IF(A182="","",TEXT(A182,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C182" s="2" t="n"/>
-      <c r="D182" s="2" t="n"/>
-      <c r="E182" s="2" t="n"/>
-      <c r="F182" s="4" t="n"/>
-      <c r="G182" s="2" t="n"/>
-      <c r="H182" s="2" t="n"/>
-      <c r="I182" s="2" t="n"/>
-    </row>
-    <row r="183">
-      <c r="A183" s="3" t="n"/>
-      <c r="B183" s="2">
-        <f>IF(A183="","",TEXT(A183,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C183" s="2" t="n"/>
-      <c r="D183" s="2" t="n"/>
-      <c r="E183" s="2" t="n"/>
-      <c r="F183" s="4" t="n"/>
-      <c r="G183" s="2" t="n"/>
-      <c r="H183" s="2" t="n"/>
-      <c r="I183" s="2" t="n"/>
-    </row>
-    <row r="184">
-      <c r="A184" s="3" t="n"/>
-      <c r="B184" s="2">
-        <f>IF(A184="","",TEXT(A184,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C184" s="2" t="n"/>
-      <c r="D184" s="2" t="n"/>
-      <c r="E184" s="2" t="n"/>
-      <c r="F184" s="4" t="n"/>
-      <c r="G184" s="2" t="n"/>
-      <c r="H184" s="2" t="n"/>
-      <c r="I184" s="2" t="n"/>
-    </row>
-    <row r="185">
-      <c r="A185" s="3" t="n"/>
-      <c r="B185" s="2">
-        <f>IF(A185="","",TEXT(A185,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C185" s="2" t="n"/>
-      <c r="D185" s="2" t="n"/>
-      <c r="E185" s="2" t="n"/>
-      <c r="F185" s="4" t="n"/>
-      <c r="G185" s="2" t="n"/>
-      <c r="H185" s="2" t="n"/>
-      <c r="I185" s="2" t="n"/>
-    </row>
-    <row r="186">
-      <c r="A186" s="3" t="n"/>
-      <c r="B186" s="2">
-        <f>IF(A186="","",TEXT(A186,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C186" s="2" t="n"/>
-      <c r="D186" s="2" t="n"/>
-      <c r="E186" s="2" t="n"/>
-      <c r="F186" s="4" t="n"/>
-      <c r="G186" s="2" t="n"/>
-      <c r="H186" s="2" t="n"/>
-      <c r="I186" s="2" t="n"/>
-    </row>
-    <row r="187">
-      <c r="A187" s="3" t="n"/>
-      <c r="B187" s="2">
-        <f>IF(A187="","",TEXT(A187,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C187" s="2" t="n"/>
-      <c r="D187" s="2" t="n"/>
-      <c r="E187" s="2" t="n"/>
-      <c r="F187" s="4" t="n"/>
-      <c r="G187" s="2" t="n"/>
-      <c r="H187" s="2" t="n"/>
-      <c r="I187" s="2" t="n"/>
-    </row>
-    <row r="188">
-      <c r="A188" s="3" t="n"/>
-      <c r="B188" s="2">
-        <f>IF(A188="","",TEXT(A188,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C188" s="2" t="n"/>
-      <c r="D188" s="2" t="n"/>
-      <c r="E188" s="2" t="n"/>
-      <c r="F188" s="4" t="n"/>
-      <c r="G188" s="2" t="n"/>
-      <c r="H188" s="2" t="n"/>
-      <c r="I188" s="2" t="n"/>
-    </row>
-    <row r="189">
-      <c r="A189" s="3" t="n"/>
-      <c r="B189" s="2">
-        <f>IF(A189="","",TEXT(A189,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C189" s="2" t="n"/>
-      <c r="D189" s="2" t="n"/>
-      <c r="E189" s="2" t="n"/>
-      <c r="F189" s="4" t="n"/>
-      <c r="G189" s="2" t="n"/>
-      <c r="H189" s="2" t="n"/>
-      <c r="I189" s="2" t="n"/>
-    </row>
-    <row r="190">
-      <c r="A190" s="3" t="n"/>
-      <c r="B190" s="2">
-        <f>IF(A190="","",TEXT(A190,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C190" s="2" t="n"/>
-      <c r="D190" s="2" t="n"/>
-      <c r="E190" s="2" t="n"/>
-      <c r="F190" s="4" t="n"/>
-      <c r="G190" s="2" t="n"/>
-      <c r="H190" s="2" t="n"/>
-      <c r="I190" s="2" t="n"/>
-    </row>
-    <row r="191">
-      <c r="A191" s="3" t="n"/>
-      <c r="B191" s="2">
-        <f>IF(A191="","",TEXT(A191,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C191" s="2" t="n"/>
-      <c r="D191" s="2" t="n"/>
-      <c r="E191" s="2" t="n"/>
-      <c r="F191" s="4" t="n"/>
-      <c r="G191" s="2" t="n"/>
-      <c r="H191" s="2" t="n"/>
-      <c r="I191" s="2" t="n"/>
-    </row>
-    <row r="192">
-      <c r="A192" s="3" t="n"/>
-      <c r="B192" s="2">
-        <f>IF(A192="","",TEXT(A192,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C192" s="2" t="n"/>
-      <c r="D192" s="2" t="n"/>
-      <c r="E192" s="2" t="n"/>
-      <c r="F192" s="4" t="n"/>
-      <c r="G192" s="2" t="n"/>
-      <c r="H192" s="2" t="n"/>
-      <c r="I192" s="2" t="n"/>
-    </row>
-    <row r="193">
-      <c r="A193" s="3" t="n"/>
-      <c r="B193" s="2">
-        <f>IF(A193="","",TEXT(A193,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C193" s="2" t="n"/>
-      <c r="D193" s="2" t="n"/>
-      <c r="E193" s="2" t="n"/>
-      <c r="F193" s="4" t="n"/>
-      <c r="G193" s="2" t="n"/>
-      <c r="H193" s="2" t="n"/>
-      <c r="I193" s="2" t="n"/>
-    </row>
-    <row r="194">
-      <c r="A194" s="3" t="n"/>
-      <c r="B194" s="2">
-        <f>IF(A194="","",TEXT(A194,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C194" s="2" t="n"/>
-      <c r="D194" s="2" t="n"/>
-      <c r="E194" s="2" t="n"/>
-      <c r="F194" s="4" t="n"/>
-      <c r="G194" s="2" t="n"/>
-      <c r="H194" s="2" t="n"/>
-      <c r="I194" s="2" t="n"/>
-    </row>
-    <row r="195">
-      <c r="A195" s="3" t="n"/>
-      <c r="B195" s="2">
-        <f>IF(A195="","",TEXT(A195,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C195" s="2" t="n"/>
-      <c r="D195" s="2" t="n"/>
-      <c r="E195" s="2" t="n"/>
-      <c r="F195" s="4" t="n"/>
-      <c r="G195" s="2" t="n"/>
-      <c r="H195" s="2" t="n"/>
-      <c r="I195" s="2" t="n"/>
-    </row>
-    <row r="196">
-      <c r="A196" s="3" t="n"/>
-      <c r="B196" s="2">
-        <f>IF(A196="","",TEXT(A196,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C196" s="2" t="n"/>
-      <c r="D196" s="2" t="n"/>
-      <c r="E196" s="2" t="n"/>
-      <c r="F196" s="4" t="n"/>
-      <c r="G196" s="2" t="n"/>
-      <c r="H196" s="2" t="n"/>
-      <c r="I196" s="2" t="n"/>
-    </row>
-    <row r="197">
-      <c r="A197" s="3" t="n"/>
-      <c r="B197" s="2">
-        <f>IF(A197="","",TEXT(A197,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C197" s="2" t="n"/>
-      <c r="D197" s="2" t="n"/>
-      <c r="E197" s="2" t="n"/>
-      <c r="F197" s="4" t="n"/>
-      <c r="G197" s="2" t="n"/>
-      <c r="H197" s="2" t="n"/>
-      <c r="I197" s="2" t="n"/>
-    </row>
-    <row r="198">
-      <c r="A198" s="3" t="n"/>
-      <c r="B198" s="2">
-        <f>IF(A198="","",TEXT(A198,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C198" s="2" t="n"/>
-      <c r="D198" s="2" t="n"/>
-      <c r="E198" s="2" t="n"/>
-      <c r="F198" s="4" t="n"/>
-      <c r="G198" s="2" t="n"/>
-      <c r="H198" s="2" t="n"/>
-      <c r="I198" s="2" t="n"/>
-    </row>
-    <row r="199">
-      <c r="A199" s="3" t="n"/>
-      <c r="B199" s="2">
-        <f>IF(A199="","",TEXT(A199,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C199" s="2" t="n"/>
-      <c r="D199" s="2" t="n"/>
-      <c r="E199" s="2" t="n"/>
-      <c r="F199" s="4" t="n"/>
-      <c r="G199" s="2" t="n"/>
-      <c r="H199" s="2" t="n"/>
-      <c r="I199" s="2" t="n"/>
-    </row>
-    <row r="200">
-      <c r="A200" s="3" t="n"/>
-      <c r="B200" s="2">
-        <f>IF(A200="","",TEXT(A200,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C200" s="2" t="n"/>
-      <c r="D200" s="2" t="n"/>
-      <c r="E200" s="2" t="n"/>
-      <c r="F200" s="4" t="n"/>
-      <c r="G200" s="2" t="n"/>
-      <c r="H200" s="2" t="n"/>
-      <c r="I200" s="2" t="n"/>
-    </row>
-    <row r="201">
-      <c r="A201" s="3" t="n"/>
-      <c r="B201" s="2">
-        <f>IF(A201="","",TEXT(A201,"MMM YYYY"))</f>
-        <v/>
-      </c>
-      <c r="C201" s="2" t="n"/>
-      <c r="D201" s="2" t="n"/>
-      <c r="E201" s="2" t="n"/>
-      <c r="F201" s="4" t="n"/>
-      <c r="G201" s="2" t="n"/>
-      <c r="H201" s="2" t="n"/>
-      <c r="I201" s="2" t="n"/>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Pre-Service</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I201"/>

</xml_diff>